<commit_message>
Updated training schedule for the 2026-2027 season.
</commit_message>
<xml_diff>
--- a/sporting-martinus/2026_2027-SPM4-trainingsschema.xlsx
+++ b/sporting-martinus/2026_2027-SPM4-trainingsschema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/siebeld/Desktop/CodingAdventures/sporting-martinus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D93B979-61CF-9A49-894D-B72873659242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1AC9C10-B1C0-E645-9E60-7B839E115E08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6960" yWindow="2160" windowWidth="28040" windowHeight="17180" xr2:uid="{0F084BDD-1696-3941-BC4E-0EF4FFF1CBE3}"/>
   </bookViews>
@@ -1112,7 +1112,7 @@
         <v>46428</v>
       </c>
       <c r="B20" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>